<commit_message>
changes for lecture 4
</commit_message>
<xml_diff>
--- a/Lecture4.RAG/eval_rag/data/evaluation_dataset.xlsx
+++ b/Lecture4.RAG/eval_rag/data/evaluation_dataset.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aleksandrmeskov/Desktop/AI evaluation/AI_practice/Lecture5/eval_rag/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aleksandrmeskov/Projects/Evaluation_AI_course_eng/Lecture4.RAG/eval_rag/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AAAB9E0-ADCA-EA44-BC3C-16314F193B9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDF00124-6C0A-C541-A63D-B816212E8C43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10360" yWindow="1720" windowWidth="28040" windowHeight="17440" xr2:uid="{BF369E15-F991-6B4A-BC00-4B14A4CF84E4}"/>
   </bookViews>
@@ -44,10 +44,10 @@
     <t>expected_response</t>
   </si>
   <si>
-    <t>расскажи о методах product_service</t>
+    <t>tell me about methods in product_service</t>
   </si>
   <si>
-    <t>как устроен процесс авторизации</t>
+    <t>how does authorization process work?</t>
   </si>
 </sst>
 </file>

</xml_diff>